<commit_message>
added emanating request template
</commit_message>
<xml_diff>
--- a/documents/excel-equivalent/1. Project Procurement Management.xlsx
+++ b/documents/excel-equivalent/1. Project Procurement Management.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patriach\Downloads\laravel\procurex\documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patriach\Downloads\laravel\procurex\documents\excel-equivalent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3FFCFB-D887-4A44-9AB1-E88BF45A0E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6175F17E-D59B-4CDE-BFAC-AC24A7E0C5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -403,30 +403,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -457,6 +433,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -466,29 +472,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -773,146 +773,146 @@
   <dimension ref="A1:R37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="12" customWidth="1"/>
-    <col min="2" max="2" width="41.5703125" style="18" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" style="12" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="27" style="13" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" style="12" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="12"/>
+    <col min="1" max="1" width="19.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="27" style="5" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
+      <c r="B1" s="6"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="8" t="s">
+      <c r="D12" s="26"/>
+      <c r="E12" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
-      <c r="O12" s="28"/>
-      <c r="P12" s="28"/>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="29"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="18"/>
+      <c r="R12" s="19"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="10" t="s">
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="K13" s="10" t="s">
+      <c r="K13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="L13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="M13" s="10" t="s">
+      <c r="M13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="N13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="O13" s="10" t="s">
+      <c r="O13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P13" s="10" t="s">
+      <c r="P13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Q13" s="10" t="s">
+      <c r="Q13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R13" s="10" t="s">
+      <c r="R13" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="11" t="s">
         <v>40</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="15">
+      <c r="E14" s="7">
         <v>130000</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="22" t="s">
         <v>49</v>
       </c>
       <c r="G14" s="1"/>
@@ -929,8 +929,8 @@
       <c r="R14" s="1"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="16" t="s">
+      <c r="A15" s="2"/>
+      <c r="B15" s="8" t="s">
         <v>41</v>
       </c>
       <c r="C15" s="1">
@@ -939,10 +939,10 @@
       <c r="D15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="9">
         <v>32000</v>
       </c>
-      <c r="F15" s="21"/>
+      <c r="F15" s="23"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -960,7 +960,7 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C16" s="1">
@@ -969,10 +969,10 @@
       <c r="D16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="9">
         <v>15000</v>
       </c>
-      <c r="F16" s="21"/>
+      <c r="F16" s="23"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
@@ -990,7 +990,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
       <c r="C17" s="1">
@@ -999,10 +999,10 @@
       <c r="D17" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="9">
         <v>35000</v>
       </c>
-      <c r="F17" s="21"/>
+      <c r="F17" s="23"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -1020,7 +1020,7 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="8" t="s">
         <v>47</v>
       </c>
       <c r="C18" s="1">
@@ -1029,10 +1029,10 @@
       <c r="D18" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="17">
+      <c r="E18" s="9">
         <v>48000</v>
       </c>
-      <c r="F18" s="22"/>
+      <c r="F18" s="24"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -1049,42 +1049,42 @@
       <c r="R18" s="1"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="23"/>
-      <c r="B19" s="24" t="s">
+      <c r="A19" s="12"/>
+      <c r="B19" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="26">
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="15">
         <v>130000</v>
       </c>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="23"/>
-      <c r="R19" s="23"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="15">
+      <c r="E20" s="7">
         <v>427000</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F20" s="22" t="s">
         <v>58</v>
       </c>
       <c r="G20" s="1"/>
@@ -1101,7 +1101,7 @@
       <c r="R20" s="1"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
+      <c r="A21" s="2"/>
       <c r="B21" t="s">
         <v>53</v>
       </c>
@@ -1111,10 +1111,10 @@
       <c r="D21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="17">
+      <c r="E21" s="9">
         <v>55000</v>
       </c>
-      <c r="F21" s="21"/>
+      <c r="F21" s="23"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -1141,10 +1141,10 @@
       <c r="D22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="9">
         <v>60000</v>
       </c>
-      <c r="F22" s="21"/>
+      <c r="F22" s="23"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -1171,10 +1171,10 @@
       <c r="D23" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="9">
         <v>138000</v>
       </c>
-      <c r="F23" s="21"/>
+      <c r="F23" s="23"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -1201,10 +1201,10 @@
       <c r="D24" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="9">
         <v>114000</v>
       </c>
-      <c r="F24" s="21"/>
+      <c r="F24" s="23"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -1231,10 +1231,10 @@
       <c r="D25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E25" s="17">
+      <c r="E25" s="9">
         <v>60000</v>
       </c>
-      <c r="F25" s="22"/>
+      <c r="F25" s="24"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -1251,72 +1251,72 @@
       <c r="R25" s="1"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="23"/>
-      <c r="B26" s="24" t="s">
+      <c r="A26" s="12"/>
+      <c r="B26" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="26">
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="15">
         <v>427000</v>
       </c>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="23"/>
-      <c r="L26" s="23"/>
-      <c r="M26" s="23"/>
-      <c r="N26" s="23"/>
-      <c r="O26" s="23"/>
-      <c r="P26" s="23"/>
-      <c r="Q26" s="23"/>
-      <c r="R26" s="23"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F33" s="12" t="s">
+      <c r="F33" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F36" s="12" t="s">
+      <c r="F36" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F37" s="12" t="s">
+      <c r="F37" s="4" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>